<commit_message>
Update KBR forecast through 2027 from August facts and tariff scenarios
</commit_message>
<xml_diff>
--- a/assets/06_2026_02_Прогноз.xlsx
+++ b/assets/06_2026_02_Прогноз.xlsx
@@ -3640,1859 +3640,1859 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:M82"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="6.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="5.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="15.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="3" width="11.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="2" width="9.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="4" width="8.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="4" width="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E1" s="5" t="n">
-        <v>46266</v>
-      </c>
-      <c r="F1" s="5" t="n">
-        <v>46266</v>
-      </c>
-      <c r="G1" s="6" t="n">
-        <v>46163</v>
-      </c>
-      <c r="H1" s="6" t="n">
-        <v>46163</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="8" t="n">
-        <v>-0.5</v>
-      </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-    </row>
-    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="n">
-        <v>44562</v>
-      </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13" t="n">
-        <v>101.22</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>108.84</v>
-      </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-    </row>
-    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="n">
-        <v>44593</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="13" t="n">
-        <v>100.94</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>108.73</v>
-      </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-    </row>
-    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="n">
-        <v>44621</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="13" t="n">
-        <v>105.55</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>113.29</v>
-      </c>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="14" t="n">
-        <f aca="false">AVERAGE($E3:$E5)^12/100^11-100</f>
-        <v>35.5951844490152</v>
-      </c>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-    </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="n">
-        <v>44652</v>
-      </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13" t="n">
-        <v>103.28</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>116</v>
-      </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="14" t="n">
-        <f aca="false">AVERAGE($E4:$E6)^12/100^11-100</f>
-        <v>46.8984496892717</v>
-      </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-    </row>
-    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="n">
-        <v>44682</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13" t="n">
-        <v>100.68</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>116.31</v>
-      </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="14" t="n">
-        <f aca="false">AVERAGE($E5:$E7)^12/100^11-100</f>
-        <v>45.4257011947349</v>
-      </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="n">
-        <v>44713</v>
-      </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18" t="n">
-        <v>99.32</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>114.88</v>
-      </c>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="14" t="n">
-        <f aca="false">AVERAGE($E6:$E8)^12/100^11-100</f>
-        <v>13.938422005549</v>
-      </c>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="n">
-        <v>44743</v>
-      </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="18" t="n">
-        <v>99.23</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>113.75</v>
-      </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="14" t="n">
-        <f aca="false">AVERAGE($E7:$E9)^12/100^11-100</f>
-        <v>-3.03689051707281</v>
-      </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="n">
-        <v>44774</v>
-      </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18" t="n">
-        <v>99.43</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>112.92</v>
-      </c>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="14" t="n">
-        <f aca="false">AVERAGE($E8:$E10)^12/100^11-100</f>
-        <v>-7.78738604247022</v>
-      </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="n">
-        <v>44805</v>
-      </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18" t="n">
-        <v>100.33</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <v>112.46</v>
-      </c>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="14" t="n">
-        <f aca="false">AVERAGE($E9:$E11)^12/100^11-100</f>
-        <v>-3.96602584605935</v>
-      </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="n">
-        <v>44835</v>
-      </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18" t="n">
-        <v>100.66</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>112.17</v>
-      </c>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="14" t="n">
-        <f aca="false">AVERAGE($E10:$E12)^12/100^11-100</f>
-        <v>1.69299655858586</v>
-      </c>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
-        <v>44866</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="18" t="n">
-        <v>100.26</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>111.51</v>
-      </c>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="14" t="n">
-        <f aca="false">AVERAGE($E11:$E13)^12/100^11-100</f>
-        <v>5.11618978817337</v>
-      </c>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="n">
-        <v>44896</v>
-      </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18" t="n">
-        <v>100.57</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>111.9</v>
-      </c>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="14" t="n">
-        <f aca="false">AVERAGE($E12:$E14)^12/100^11-100</f>
-        <v>6.12553306065077</v>
-      </c>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
-        <v>44927</v>
-      </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="18" t="n">
-        <v>101.13</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <v>111.8</v>
-      </c>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="14" t="n">
-        <f aca="false">AVERAGE($E13:$E15)^12/100^11-100</f>
-        <v>8.12794364790587</v>
-      </c>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="n">
-        <v>44958</v>
-      </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="20" t="n">
-        <v>100.75</v>
-      </c>
-      <c r="F16" s="20" t="n">
-        <v>111.59</v>
-      </c>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="14" t="n">
-        <f aca="false">AVERAGE($E14:$E16)^12/100^11-100</f>
-        <v>10.2523891898909</v>
-      </c>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
-        <v>44986</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="21" t="n">
-        <v>100.39</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <v>106.14</v>
-      </c>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="14" t="n">
-        <f aca="false">AVERAGE($E15:$E17)^12/100^11-100</f>
-        <v>9.46757453632417</v>
-      </c>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="n">
-        <v>45017</v>
-      </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="22" t="n">
-        <v>100.72</v>
-      </c>
-      <c r="F18" s="20" t="n">
-        <v>103.51</v>
-      </c>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="14" t="n">
-        <f aca="false">AVERAGE($E16:$E18)^12/100^11-100</f>
-        <v>7.69902108971681</v>
-      </c>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
-        <v>45047</v>
-      </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="22" t="n">
-        <v>99.75</v>
-      </c>
-      <c r="F19" s="20" t="n">
-        <v>102.55</v>
-      </c>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="14" t="n">
-        <f aca="false">AVERAGE($E17:$E19)^12/100^11-100</f>
-        <v>3.49475895939679</v>
-      </c>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="n">
-        <v>45078</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="22" t="n">
-        <v>100.43</v>
-      </c>
-      <c r="F20" s="20" t="n">
-        <v>103.69</v>
-      </c>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="14" t="n">
-        <f aca="false">AVERAGE($E18:$E20)^12/100^11-100</f>
-        <v>3.65999802881309</v>
-      </c>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
-        <v>45108</v>
-      </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="22" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="F21" s="20" t="n">
-        <v>105.03</v>
-      </c>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="14" t="n">
-        <f aca="false">AVERAGE($E19:$E21)^12/100^11-100</f>
-        <v>2.75416684857622</v>
-      </c>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="n">
-        <v>45139</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="22" t="n">
-        <v>99.93</v>
-      </c>
-      <c r="F22" s="20" t="n">
-        <v>105.56</v>
-      </c>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="14" t="n">
-        <f aca="false">AVERAGE($E20:$E22)^12/100^11-100</f>
-        <v>3.49475895939679</v>
-      </c>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="25"/>
-    </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="n">
-        <v>45170</v>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="22" t="n">
-        <v>101.75</v>
-      </c>
-      <c r="F23" s="20" t="n">
-        <v>107.05</v>
-      </c>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="14" t="n">
-        <f aca="false">AVERAGE($E21:$E23)^12/100^11-100</f>
-        <v>9.07709064358237</v>
-      </c>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="25"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="n">
-        <v>45200</v>
-      </c>
-      <c r="B24" s="24" t="n">
-        <f aca="false">E24-0.5</f>
-        <v>99.96</v>
-      </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="22" t="n">
-        <v>100.46</v>
-      </c>
-      <c r="F24" s="20" t="n">
-        <v>106.84</v>
-      </c>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="14" t="n">
-        <f aca="false">AVERAGE($E22:$E24)^12/100^11-100</f>
-        <v>8.90395244059377</v>
-      </c>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-    </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="n">
-        <v>45231</v>
-      </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="22" t="n">
-        <v>100.74</v>
-      </c>
-      <c r="F25" s="20" t="n">
-        <v>107.34</v>
-      </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="14" t="n">
-        <f aca="false">AVERAGE($E23:$E25)^12/100^11-100</f>
-        <v>12.4595717465677</v>
-      </c>
-      <c r="J25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="25"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="n">
-        <v>45261</v>
-      </c>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="22" t="n">
-        <v>100.29</v>
-      </c>
-      <c r="F26" s="20" t="n">
-        <v>107.05</v>
-      </c>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="14" t="n">
-        <f aca="false">AVERAGE($E24:$E26)^12/100^11-100</f>
-        <v>6.12553306065077</v>
-      </c>
-      <c r="J26" s="25"/>
-      <c r="K26" s="25"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="n">
-        <v>45292</v>
-      </c>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="22" t="n">
-        <v>100.87</v>
-      </c>
-      <c r="F27" s="20" t="n">
-        <v>106.77</v>
-      </c>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="14" t="n">
-        <f aca="false">AVERAGE($E25:$E27)^12/100^11-100</f>
-        <v>7.87040260177953</v>
-      </c>
-      <c r="J27" s="25"/>
-      <c r="K27" s="25"/>
-      <c r="L27" s="25"/>
-      <c r="M27" s="25"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="n">
-        <v>45323</v>
-      </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="22" t="n">
-        <v>100.53</v>
-      </c>
-      <c r="F28" s="20" t="n">
-        <v>106.54</v>
-      </c>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="14" t="n">
-        <f aca="false">AVERAGE($E26:$E28)^12/100^11-100</f>
-        <v>6.97343059130941</v>
-      </c>
-      <c r="J28" s="25"/>
-      <c r="K28" s="25"/>
-      <c r="L28" s="25"/>
-      <c r="M28" s="25"/>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="n">
-        <v>45352</v>
-      </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="22" t="n">
-        <v>100.53</v>
-      </c>
-      <c r="F29" s="20" t="n">
-        <v>106.68</v>
-      </c>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="14" t="n">
-        <f aca="false">AVERAGE($E27:$E29)^12/100^11-100</f>
-        <v>7.99910275378316</v>
-      </c>
-      <c r="J29" s="25"/>
-      <c r="K29" s="25"/>
-      <c r="L29" s="25"/>
-      <c r="M29" s="25"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="n">
-        <v>45383</v>
-      </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="21" t="n">
-        <v>100.38</v>
-      </c>
-      <c r="F30" s="20" t="n">
-        <v>106.32</v>
-      </c>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="14" t="n">
-        <f aca="false">AVERAGE($E28:$E30)^12/100^11-100</f>
-        <v>5.91452350359876</v>
-      </c>
-      <c r="J30" s="25"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="25"/>
-      <c r="M30" s="25"/>
-    </row>
-    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="n">
-        <v>45413</v>
-      </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="21" t="n">
-        <v>100.94</v>
-      </c>
-      <c r="F31" s="20" t="n">
-        <v>107.59</v>
-      </c>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="14" t="n">
-        <f aca="false">AVERAGE($E29:$E31)^12/100^11-100</f>
-        <v>7.65621472911278</v>
-      </c>
-      <c r="J31" s="25"/>
-      <c r="K31" s="25"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="25"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="n">
-        <v>45444</v>
-      </c>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="21" t="n">
-        <v>100.18</v>
-      </c>
-      <c r="F32" s="20" t="n">
-        <v>107.33</v>
-      </c>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="14" t="n">
-        <f aca="false">AVERAGE($E30:$E32)^12/100^11-100</f>
-        <v>6.16778118644996</v>
-      </c>
-      <c r="J32" s="25"/>
-      <c r="K32" s="25"/>
-      <c r="L32" s="25"/>
-      <c r="M32" s="25"/>
-    </row>
-    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="n">
-        <v>45474</v>
-      </c>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="21" t="n">
-        <v>101.07</v>
-      </c>
-      <c r="F33" s="20" t="n">
-        <v>107.94</v>
-      </c>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="14" t="n">
-        <f aca="false">AVERAGE($E31:$E33)^12/100^11-100</f>
-        <v>9.12041460123689</v>
-      </c>
-      <c r="J33" s="25"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="n">
-        <v>45505</v>
-      </c>
-      <c r="B34" s="24"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="22" t="n">
-        <v>100.09</v>
-      </c>
-      <c r="F34" s="20" t="n">
-        <v>108.1</v>
-      </c>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="14" t="n">
-        <f aca="false">AVERAGE($E32:$E34)^12/100^11-100</f>
-        <v>5.49365770738656</v>
-      </c>
-      <c r="J34" s="25"/>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="25"/>
-    </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="n">
-        <v>45536</v>
-      </c>
-      <c r="B35" s="24"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="21" t="n">
-        <v>100.62</v>
-      </c>
-      <c r="F35" s="20" t="n">
-        <v>106.91</v>
-      </c>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="14" t="n">
-        <f aca="false">AVERAGE($E33:$E35)^12/100^11-100</f>
-        <v>7.35700662123239</v>
-      </c>
-      <c r="J35" s="25"/>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-    </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="n">
-        <v>45566</v>
-      </c>
-      <c r="B36" s="24"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="22" t="n">
-        <v>101.02</v>
-      </c>
-      <c r="F36" s="20" t="n">
-        <v>107.49</v>
-      </c>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="14" t="n">
-        <f aca="false">AVERAGE($E34:$E36)^12/100^11-100</f>
-        <v>7.14375346230894</v>
-      </c>
-      <c r="J36" s="25"/>
-      <c r="K36" s="25"/>
-      <c r="L36" s="25"/>
-      <c r="M36" s="25"/>
-    </row>
-    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="27" t="n">
-        <v>45597</v>
-      </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="29" t="n">
-        <v>101.5</v>
-      </c>
-      <c r="F37" s="30" t="n">
-        <v>108.31</v>
-      </c>
-      <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="14" t="n">
-        <f aca="false">AVERAGE($E35:$E37)^12/100^11-100</f>
-        <v>13.3088674453934</v>
-      </c>
-      <c r="J37" s="25"/>
-      <c r="K37" s="25"/>
-      <c r="L37" s="25"/>
-      <c r="M37" s="25"/>
-    </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="16" t="n">
-        <v>45627</v>
-      </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="22" t="n">
-        <v>100.91</v>
-      </c>
-      <c r="F38" s="20" t="n">
-        <v>108.98</v>
-      </c>
-      <c r="G38" s="32"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="24" t="n">
-        <f aca="false">AVERAGE($E36:$E38)^12/100^11-100</f>
-        <v>14.616501588559</v>
-      </c>
-      <c r="J38" s="25"/>
-      <c r="K38" s="25"/>
-      <c r="L38" s="25"/>
-      <c r="M38" s="25"/>
-    </row>
-    <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33" t="n">
-        <v>45658</v>
-      </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="22" t="n">
-        <v>100.84</v>
-      </c>
-      <c r="F39" s="22" t="n">
-        <v>108.95</v>
-      </c>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="34" t="n">
-        <f aca="false">AVERAGE($E37:$E39)^12/100^11-100</f>
-        <v>13.8032481613878</v>
-      </c>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
-    </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="35" t="n">
-        <v>45689</v>
-      </c>
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="34"/>
-      <c r="E40" s="22" t="n">
-        <v>101.34</v>
-      </c>
-      <c r="F40" s="22" t="n">
-        <v>109.83</v>
-      </c>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
-      <c r="I40" s="34" t="n">
-        <f aca="false">AVERAGE($E38:$E40)^12/100^11-100</f>
-        <v>13.0848004136226</v>
-      </c>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="36" t="n">
-        <v>45717</v>
-      </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="29" t="n">
-        <v>100.81</v>
-      </c>
-      <c r="F41" s="29" t="n">
-        <v>110.13</v>
-      </c>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="37" t="n">
-        <f aca="false">AVERAGE($E39:$E41)^12/100^11-100</f>
-        <v>12.6378843790016</v>
-      </c>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
-      <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="39" t="n">
-        <v>45748</v>
-      </c>
-      <c r="B42" s="40"/>
-      <c r="C42" s="40"/>
-      <c r="D42" s="40"/>
-      <c r="E42" s="41" t="n">
-        <v>100.53</v>
-      </c>
-      <c r="F42" s="41" t="n">
-        <v>110.3</v>
-      </c>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="40" t="n">
-        <f aca="false">AVERAGE($E40:$E42)^12/100^11-100</f>
-        <v>11.2627133732496</v>
-      </c>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-    </row>
-    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="43" t="n">
-        <v>45778</v>
-      </c>
-      <c r="B43" s="44"/>
-      <c r="C43" s="44"/>
-      <c r="D43" s="44"/>
-      <c r="E43" s="45" t="n">
-        <v>99.93</v>
-      </c>
-      <c r="F43" s="45" t="n">
-        <v>109.2</v>
-      </c>
-      <c r="G43" s="46"/>
-      <c r="H43" s="46"/>
-      <c r="I43" s="44" t="n">
-        <f aca="false">AVERAGE($E41:$E43)^12/100^11-100</f>
-        <v>5.19996439209056</v>
-      </c>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="3"/>
-      <c r="M43" s="3"/>
-    </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="35" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="34"/>
-      <c r="E44" s="22" t="n">
-        <v>99.96</v>
-      </c>
-      <c r="F44" s="22" t="n">
-        <v>108.96</v>
-      </c>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="34" t="n">
-        <f aca="false">AVERAGE($E42:$E44)^12/100^11-100</f>
-        <v>1.69299655858586</v>
-      </c>
-      <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-      <c r="M44" s="3"/>
-    </row>
-    <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="33" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B45" s="34"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="34"/>
-      <c r="E45" s="22" t="n">
-        <v>100.36</v>
-      </c>
-      <c r="F45" s="22" t="n">
-        <v>108.19</v>
-      </c>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="34" t="n">
-        <f aca="false">AVERAGE($E43:$E45)^12/100^11-100</f>
-        <v>1.00459608871815</v>
-      </c>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-      <c r="L45" s="14"/>
-      <c r="M45" s="14"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="35" t="n">
-        <v>45870</v>
-      </c>
-      <c r="B46" s="34"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="22" t="n">
-        <v>99.43</v>
-      </c>
-      <c r="F46" s="22" t="n">
-        <v>107.48</v>
-      </c>
-      <c r="G46" s="32"/>
-      <c r="H46" s="32"/>
-      <c r="I46" s="34" t="n">
-        <f aca="false">AVERAGE($E44:$E46)^12/100^11-100</f>
-        <v>-0.995429374308358</v>
-      </c>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-    </row>
-    <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="33" t="n">
-        <v>45901</v>
-      </c>
-      <c r="B47" s="34"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="34"/>
-      <c r="E47" s="22" t="n">
-        <v>101</v>
-      </c>
-      <c r="F47" s="22" t="n">
-        <v>107.88</v>
-      </c>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="34" t="n">
-        <f aca="false">AVERAGE($E45:$E47)^12/100^11-100</f>
-        <v>3.20617145915737</v>
-      </c>
-      <c r="J47" s="14"/>
-      <c r="K47" s="14"/>
-      <c r="L47" s="14"/>
-      <c r="M47" s="14"/>
-    </row>
-    <row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="35" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B48" s="34"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="34"/>
-      <c r="E48" s="22" t="n">
-        <v>100.53</v>
-      </c>
-      <c r="F48" s="22" t="n">
-        <v>107.36</v>
-      </c>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="34" t="n">
-        <f aca="false">AVERAGE($E46:$E48)^12/100^11-100</f>
-        <v>3.90831011312588</v>
-      </c>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="36" t="n">
-        <v>45962</v>
-      </c>
-      <c r="B49" s="37"/>
-      <c r="C49" s="34"/>
-      <c r="D49" s="34"/>
-      <c r="E49" s="29" t="n">
-        <v>100.15</v>
-      </c>
-      <c r="F49" s="29" t="n">
-        <v>105.93</v>
-      </c>
-      <c r="G49" s="38"/>
-      <c r="H49" s="38"/>
-      <c r="I49" s="37" t="n">
-        <f aca="false">AVERAGE($E47:$E49)^12/100^11-100</f>
-        <v>6.93088867179823</v>
-      </c>
-      <c r="J49" s="14"/>
-      <c r="K49" s="14"/>
-      <c r="L49" s="14"/>
-      <c r="M49" s="14"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="39" t="n">
-        <v>45992</v>
-      </c>
-      <c r="B50" s="40"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="34"/>
-      <c r="E50" s="41" t="n">
-        <v>100.29</v>
-      </c>
-      <c r="F50" s="41" t="n">
-        <v>105.28</v>
-      </c>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="40" t="n">
-        <f aca="false">AVERAGE($E48:$E50)^12/100^11-100</f>
-        <v>3.94974843103184</v>
-      </c>
-      <c r="J50" s="14"/>
-      <c r="K50" s="14"/>
-      <c r="L50" s="14"/>
-      <c r="M50" s="14"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="43" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B51" s="47"/>
-      <c r="C51" s="34" t="n">
-        <f aca="false">E51-100</f>
-        <v>1.59999999999999</v>
-      </c>
-      <c r="D51" s="34" t="n">
-        <f aca="false">F51-100</f>
-        <v>6.06999999999999</v>
-      </c>
-      <c r="E51" s="44" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="F51" s="44" t="n">
-        <f aca="false">ROUND(PRODUCT(E40:E51)/100^11,2)</f>
-        <v>106.07</v>
-      </c>
-      <c r="G51" s="48" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="H51" s="48" t="n">
-        <v>106.07</v>
-      </c>
-      <c r="I51" s="40" t="n">
-        <f aca="false">AVERAGE($E49:$E51)^12/100^11-100</f>
-        <v>8.4722085025155</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="35" t="n">
-        <v>46054</v>
-      </c>
-      <c r="B52" s="26"/>
-      <c r="C52" s="34" t="n">
-        <f aca="false">E52-100</f>
-        <v>1.09999999999999</v>
-      </c>
-      <c r="D52" s="34" t="n">
-        <f aca="false">F52-100</f>
-        <v>5.81999999999999</v>
-      </c>
-      <c r="E52" s="34" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="F52" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E41:E52)/100^11,2)</f>
-        <v>105.82</v>
-      </c>
-      <c r="G52" s="49" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="H52" s="49" t="n">
-        <v>105.82</v>
-      </c>
-      <c r="I52" s="40" t="n">
-        <f aca="false">AVERAGE($E50:$E52)^12/100^11-100</f>
-        <v>12.6378843790016</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="33" t="n">
-        <v>46082</v>
-      </c>
-      <c r="B53" s="26"/>
-      <c r="C53" s="34" t="n">
-        <f aca="false">E53-100</f>
-        <v>0.540000000000006</v>
-      </c>
-      <c r="D53" s="34" t="n">
-        <f aca="false">F53-100</f>
-        <v>5.54000000000001</v>
-      </c>
-      <c r="E53" s="50" t="n">
-        <v>100.54</v>
-      </c>
-      <c r="F53" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E42:E53)/100^11,2)</f>
-        <v>105.54</v>
-      </c>
-      <c r="G53" s="49" t="n">
-        <v>100.54</v>
-      </c>
-      <c r="H53" s="49" t="n">
-        <v>105.54</v>
-      </c>
-      <c r="I53" s="40" t="n">
-        <f aca="false">AVERAGE($E51:$E53)^12/100^11-100</f>
-        <v>13.7582228911073</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="35" t="n">
-        <v>46113</v>
-      </c>
-      <c r="B54" s="26"/>
-      <c r="C54" s="34" t="n">
-        <f aca="false">E54-100</f>
-        <v>-0.280000000000001</v>
-      </c>
-      <c r="D54" s="34" t="n">
-        <f aca="false">F54-100</f>
-        <v>4.69</v>
-      </c>
-      <c r="E54" s="34" t="n">
-        <v>99.72</v>
-      </c>
-      <c r="F54" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E43:E54)/100^11,2)</f>
-        <v>104.69</v>
-      </c>
-      <c r="G54" s="49" t="n">
-        <v>99.72</v>
-      </c>
-      <c r="H54" s="49" t="n">
-        <v>104.69</v>
-      </c>
-      <c r="I54" s="40" t="n">
-        <f aca="false">AVERAGE($E52:$E54)^12/100^11-100</f>
-        <v>5.57770802282748</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="33" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B55" s="51"/>
-      <c r="C55" s="34" t="n">
-        <f aca="false">E55-100</f>
-        <v>0.0900000000000034</v>
-      </c>
-      <c r="D55" s="34" t="n">
-        <f aca="false">F55-100</f>
-        <v>4.84999999999999</v>
-      </c>
-      <c r="E55" s="34" t="n">
-        <v>100.09</v>
-      </c>
-      <c r="F55" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E44:E55)/100^11,2)</f>
-        <v>104.85</v>
-      </c>
-      <c r="G55" s="49" t="n">
-        <v>99.9</v>
-      </c>
-      <c r="H55" s="49" t="n">
-        <v>104.66</v>
-      </c>
-      <c r="I55" s="40" t="n">
-        <f aca="false">AVERAGE($E53:$E55)^12/100^11-100</f>
-        <v>1.4090183603949</v>
-      </c>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
-      <c r="M55" s="52"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="35" t="n">
-        <v>46174</v>
-      </c>
-      <c r="B56" s="26"/>
-      <c r="C56" s="34" t="n">
-        <f aca="false">E56-100</f>
-        <v>1.06</v>
-      </c>
-      <c r="D56" s="34" t="n">
-        <f aca="false">F56-100</f>
-        <v>6.01000000000001</v>
-      </c>
-      <c r="E56" s="34" t="n">
-        <v>101.06</v>
-      </c>
-      <c r="F56" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E45:E56)/100^11,2)</f>
-        <v>106.01</v>
-      </c>
-      <c r="G56" s="49" t="n">
-        <v>100</v>
-      </c>
-      <c r="H56" s="49" t="n">
-        <v>104.7</v>
-      </c>
-      <c r="I56" s="40" t="n">
-        <f aca="false">AVERAGE($E54:$E56)^12/100^11-100</f>
-        <v>3.53604607534096</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="33" t="n">
-        <v>46204</v>
-      </c>
-      <c r="B57" s="53"/>
-      <c r="C57" s="34" t="n">
-        <f aca="false">E57-100</f>
-        <v>1.40000000000001</v>
-      </c>
-      <c r="D57" s="34" t="n">
-        <f aca="false">F57-100</f>
-        <v>7.11</v>
-      </c>
-      <c r="E57" s="34" t="n">
-        <v>101.4</v>
-      </c>
-      <c r="F57" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E46:E57)/100^11,2)</f>
-        <v>107.11</v>
-      </c>
-      <c r="G57" s="49" t="n">
-        <v>99.9</v>
-      </c>
-      <c r="H57" s="49" t="n">
-        <v>104.22</v>
-      </c>
-      <c r="I57" s="40" t="n">
-        <f aca="false">AVERAGE($E55:$E57)^12/100^11-100</f>
-        <v>10.6906226923438</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="35" t="n">
-        <v>46235</v>
-      </c>
-      <c r="B58" s="53"/>
-      <c r="C58" s="53"/>
-      <c r="D58" s="53"/>
-      <c r="E58" s="50" t="n">
-        <v>100</v>
-      </c>
-      <c r="F58" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E47:E58)/100^11,2)</f>
-        <v>107.72</v>
-      </c>
-      <c r="G58" s="49" t="n">
-        <v>99.85</v>
-      </c>
-      <c r="H58" s="49" t="n">
-        <v>104.66</v>
-      </c>
-      <c r="I58" s="40" t="n">
-        <f aca="false">AVERAGE($E56:$E58)^12/100^11-100</f>
-        <v>10.2961408608195</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="33" t="n">
-        <v>46266</v>
-      </c>
-      <c r="B59" s="53"/>
-      <c r="C59" s="53"/>
-      <c r="D59" s="53"/>
-      <c r="E59" s="50" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="F59" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E48:E59)/100^11,2)</f>
-        <v>107.19</v>
-      </c>
-      <c r="G59" s="49" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="H59" s="49" t="n">
-        <v>104.09</v>
-      </c>
-      <c r="I59" s="40" t="n">
-        <f aca="false">AVERAGE($E57:$E59)^12/100^11-100</f>
-        <v>7.87040260177953</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="35" t="n">
-        <v>46296</v>
-      </c>
-      <c r="B60" s="26"/>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="E60" s="50" t="n">
-        <v>101.3</v>
-      </c>
-      <c r="F60" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E49:E60)/100^11,2)</f>
-        <v>108.01</v>
-      </c>
-      <c r="G60" s="49" t="n">
-        <v>101.3</v>
-      </c>
-      <c r="H60" s="49" t="n">
-        <v>104.88</v>
-      </c>
-      <c r="I60" s="40" t="n">
-        <f aca="false">AVERAGE($E58:$E60)^12/100^11-100</f>
-        <v>7.44241677219257</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="33" t="n">
-        <v>46327</v>
-      </c>
-      <c r="B61" s="26"/>
-      <c r="C61" s="26"/>
-      <c r="D61" s="26"/>
-      <c r="E61" s="50" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="F61" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E50:E61)/100^11,2)</f>
-        <v>108.33</v>
-      </c>
-      <c r="G61" s="49" t="n">
-        <v>100.3</v>
-      </c>
-      <c r="H61" s="49" t="n">
-        <v>105.04</v>
-      </c>
-      <c r="I61" s="40" t="n">
-        <f aca="false">AVERAGE($E59:$E61)^12/100^11-100</f>
-        <v>9.38068976709832</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="35" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="26"/>
-      <c r="E62" s="50" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="F62" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E51:E62)/100^11,2)</f>
-        <v>108.56</v>
-      </c>
-      <c r="G62" s="49" t="n">
-        <v>100.35</v>
-      </c>
-      <c r="H62" s="49" t="n">
-        <v>105.1</v>
-      </c>
-      <c r="I62" s="40" t="n">
-        <f aca="false">AVERAGE($E60:$E62)^12/100^11-100</f>
-        <v>9.38068976709832</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="33" t="n">
-        <v>46388</v>
-      </c>
-      <c r="E63" s="25" t="n">
-        <v>100.9</v>
-      </c>
-      <c r="F63" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E52:E63)/100^11,2)</f>
-        <v>107.81</v>
-      </c>
-      <c r="G63" s="54" t="n">
-        <v>100.95</v>
-      </c>
-      <c r="H63" s="54" t="n">
-        <v>104.43</v>
-      </c>
-      <c r="I63" s="25"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="35" t="n">
-        <v>46419</v>
-      </c>
-      <c r="E64" s="25" t="n">
-        <v>100.65</v>
-      </c>
-      <c r="F64" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E53:E64)/100^11,2)</f>
-        <v>107.33</v>
-      </c>
-      <c r="G64" s="54" t="n">
-        <v>100.65</v>
-      </c>
-      <c r="H64" s="54" t="n">
-        <v>103.97</v>
-      </c>
-      <c r="I64" s="25"/>
-    </row>
-    <row r="65" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="33" t="n">
-        <v>46447</v>
-      </c>
-      <c r="E65" s="25" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="F65" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E54:E65)/100^11,2)</f>
-        <v>107.29</v>
-      </c>
-      <c r="G65" s="54" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="H65" s="54" t="n">
-        <v>103.93</v>
-      </c>
-      <c r="I65" s="25"/>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="35" t="n">
-        <v>46478</v>
-      </c>
-      <c r="E66" s="25" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="F66" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E55:E66)/100^11,2)</f>
-        <v>108.07</v>
-      </c>
-      <c r="G66" s="54" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="H66" s="54" t="n">
-        <v>104.69</v>
-      </c>
-      <c r="I66" s="25"/>
-    </row>
-    <row r="67" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="33" t="n">
-        <v>46508</v>
-      </c>
-      <c r="E67" s="25" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="F67" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E56:E67)/100^11,2)</f>
-        <v>108.19</v>
-      </c>
-      <c r="G67" s="54" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="H67" s="54" t="n">
-        <v>105</v>
-      </c>
-      <c r="I67" s="25"/>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="35" t="n">
-        <v>46539</v>
-      </c>
-      <c r="E68" s="25" t="n">
-        <v>100.15</v>
-      </c>
-      <c r="F68" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E57:E68)/100^11,2)</f>
-        <v>107.22</v>
-      </c>
-      <c r="G68" s="54" t="n">
-        <v>100.1</v>
-      </c>
-      <c r="H68" s="54" t="n">
-        <v>105.11</v>
-      </c>
-      <c r="I68" s="25"/>
-    </row>
-    <row r="69" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="33" t="n">
-        <v>46569</v>
-      </c>
-      <c r="E69" s="25" t="n">
-        <v>100.05</v>
-      </c>
-      <c r="F69" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E58:E69)/100^11,2)</f>
-        <v>105.79</v>
-      </c>
-      <c r="G69" s="54" t="n">
-        <v>100.05</v>
-      </c>
-      <c r="H69" s="54" t="n">
-        <v>105.26</v>
-      </c>
-      <c r="I69" s="25"/>
-    </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="35" t="n">
-        <v>46600</v>
-      </c>
-      <c r="E70" s="25" t="n">
-        <v>99.95</v>
-      </c>
-      <c r="F70" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E59:E70)/100^11,2)</f>
-        <v>105.74</v>
-      </c>
-      <c r="G70" s="54" t="n">
-        <v>99.95</v>
-      </c>
-      <c r="H70" s="54" t="n">
-        <v>105.37</v>
-      </c>
-      <c r="I70" s="25"/>
-    </row>
-    <row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="33" t="n">
-        <v>46631</v>
-      </c>
-      <c r="E71" s="25" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="F71" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E60:E71)/100^11,2)</f>
-        <v>105.69</v>
-      </c>
-      <c r="G71" s="54" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="H71" s="54" t="n">
-        <v>105.37</v>
-      </c>
-      <c r="I71" s="25"/>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="35" t="n">
-        <v>46661</v>
-      </c>
-      <c r="E72" s="25" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="F72" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E61:E72)/100^11,2)</f>
-        <v>104.8</v>
-      </c>
-      <c r="G72" s="54" t="n">
-        <v>100.45</v>
-      </c>
-      <c r="H72" s="54" t="n">
-        <v>104.49</v>
-      </c>
-      <c r="I72" s="25"/>
-    </row>
-    <row r="73" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="33" t="n">
-        <v>46692</v>
-      </c>
-      <c r="E73" s="25" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="F73" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E62:E73)/100^11,2)</f>
-        <v>104.54</v>
-      </c>
-      <c r="G73" s="54" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="H73" s="54" t="n">
-        <v>104.38</v>
-      </c>
-      <c r="I73" s="25"/>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="35" t="n">
-        <v>46722</v>
-      </c>
-      <c r="E74" s="25" t="n">
-        <v>100</v>
-      </c>
-      <c r="F74" s="34" t="n">
-        <f aca="false">ROUND(PRODUCT(E63:E74)/100^11,2)</f>
-        <v>104.02</v>
-      </c>
-      <c r="G74" s="54" t="n">
-        <v>100</v>
-      </c>
-      <c r="H74" s="54" t="n">
-        <v>104.02</v>
-      </c>
-      <c r="I74" s="25"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="55"/>
-      <c r="E75" s="56"/>
-      <c r="F75" s="25"/>
-      <c r="G75" s="54"/>
-      <c r="H75" s="54"/>
-      <c r="I75" s="25"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="55"/>
-      <c r="E76" s="56"/>
-      <c r="F76" s="25"/>
-      <c r="G76" s="54"/>
-      <c r="H76" s="54"/>
-      <c r="I76" s="25"/>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="55"/>
-      <c r="E77" s="56"/>
-      <c r="F77" s="25"/>
-      <c r="G77" s="54"/>
-      <c r="H77" s="54"/>
-      <c r="I77" s="25"/>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="55"/>
-      <c r="E78" s="56"/>
-      <c r="F78" s="25"/>
-      <c r="G78" s="54"/>
-      <c r="H78" s="54"/>
-      <c r="I78" s="25"/>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="55"/>
-      <c r="E79" s="56"/>
-      <c r="F79" s="25"/>
-      <c r="G79" s="54"/>
-      <c r="H79" s="54"/>
-      <c r="I79" s="25"/>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G81" s="14"/>
-      <c r="H81" s="14"/>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G82" s="14"/>
-      <c r="H82" s="14"/>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="J23:M24">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max" val="0"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr filterMode="false">
+    <ns0:pageSetUpPr fitToPage="false"/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:M82"/>
+  <ns0:sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <ns0:cols>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.9"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="6.4"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="5.09"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="15.29"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="3" width="11.1"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="2" width="9.9"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="6.7"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="10" style="4" width="8.4"/>
+    <ns0:col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="4" width="12"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="E1" s="5" t="n">
+        <ns0:v>46266</ns0:v>
+      </ns0:c>
+      <ns0:c r="F1" s="5" t="n">
+        <ns0:v>46266</ns0:v>
+      </ns0:c>
+      <ns0:c r="G1" s="6" t="n">
+        <ns0:v>46163</ns0:v>
+      </ns0:c>
+      <ns0:c r="H1" s="6" t="n">
+        <ns0:v>46163</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A2" s="7" t="s">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="8" t="n">
+        <ns0:v>-0.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="8"/>
+      <ns0:c r="D2" s="8"/>
+      <ns0:c r="E2" s="7" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="F2" s="7" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G2" s="8" t="s">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H2" s="8" t="s">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="I2" s="9" t="s">
+        <ns0:v>3</ns0:v>
+      </ns0:c>
+      <ns0:c r="J2" s="10"/>
+      <ns0:c r="K2" s="10"/>
+      <ns0:c r="L2" s="10"/>
+      <ns0:c r="M2" s="10"/>
+    </ns0:row>
+    <ns0:row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A3" s="11" t="n">
+        <ns0:v>44562</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" s="12"/>
+      <ns0:c r="C3" s="12"/>
+      <ns0:c r="D3" s="12"/>
+      <ns0:c r="E3" s="13">
+        <ns0:v>101.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="F3" s="13">
+        <ns0:v>108.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="G3" s="12"/>
+      <ns0:c r="H3" s="12"/>
+      <ns0:c r="I3" s="14"/>
+      <ns0:c r="J3" s="15"/>
+      <ns0:c r="K3" s="15"/>
+      <ns0:c r="L3" s="15"/>
+      <ns0:c r="M3" s="15"/>
+    </ns0:row>
+    <ns0:row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A4" s="16" t="n">
+        <ns0:v>44593</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="12"/>
+      <ns0:c r="C4" s="12"/>
+      <ns0:c r="D4" s="12"/>
+      <ns0:c r="E4" s="13">
+        <ns0:v>100.94</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="13">
+        <ns0:v>108.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="12"/>
+      <ns0:c r="H4" s="12"/>
+      <ns0:c r="I4" s="14"/>
+      <ns0:c r="J4" s="15"/>
+      <ns0:c r="K4" s="15"/>
+      <ns0:c r="L4" s="15"/>
+      <ns0:c r="M4" s="15"/>
+    </ns0:row>
+    <ns0:row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A5" s="11" t="n">
+        <ns0:v>44621</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" s="12"/>
+      <ns0:c r="C5" s="12"/>
+      <ns0:c r="D5" s="12"/>
+      <ns0:c r="E5" s="13">
+        <ns0:v>105.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" s="13">
+        <ns0:v>113.27</ns0:v>
+      </ns0:c>
+      <ns0:c r="G5" s="12"/>
+      <ns0:c r="H5" s="12"/>
+      <ns0:c r="I5" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E3:$E5)^12/100^11-100</ns0:f>
+        <ns0:v>35.5951844490152</ns0:v>
+      </ns0:c>
+      <ns0:c r="J5" s="15"/>
+      <ns0:c r="K5" s="15"/>
+      <ns0:c r="L5" s="15"/>
+      <ns0:c r="M5" s="15"/>
+    </ns0:row>
+    <ns0:row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A6" s="16" t="n">
+        <ns0:v>44652</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" s="12"/>
+      <ns0:c r="C6" s="12"/>
+      <ns0:c r="D6" s="12"/>
+      <ns0:c r="E6" s="13">
+        <ns0:v>103.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="F6" s="13">
+        <ns0:v>115.99</ns0:v>
+      </ns0:c>
+      <ns0:c r="G6" s="12"/>
+      <ns0:c r="H6" s="12"/>
+      <ns0:c r="I6" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E4:$E6)^12/100^11-100</ns0:f>
+        <ns0:v>46.8984496892717</ns0:v>
+      </ns0:c>
+      <ns0:c r="J6" s="15"/>
+      <ns0:c r="K6" s="15"/>
+      <ns0:c r="L6" s="15"/>
+      <ns0:c r="M6" s="15"/>
+    </ns0:row>
+    <ns0:row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A7" s="11" t="n">
+        <ns0:v>44682</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" s="12"/>
+      <ns0:c r="C7" s="12"/>
+      <ns0:c r="D7" s="12"/>
+      <ns0:c r="E7" s="13">
+        <ns0:v>100.68</ns0:v>
+      </ns0:c>
+      <ns0:c r="F7" s="13">
+        <ns0:v>116.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="G7" s="12"/>
+      <ns0:c r="H7" s="12"/>
+      <ns0:c r="I7" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E5:$E7)^12/100^11-100</ns0:f>
+        <ns0:v>45.4257011947349</ns0:v>
+      </ns0:c>
+      <ns0:c r="J7" s="3"/>
+      <ns0:c r="K7" s="3"/>
+      <ns0:c r="L7" s="3"/>
+      <ns0:c r="M7" s="3"/>
+    </ns0:row>
+    <ns0:row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A8" s="16" t="n">
+        <ns0:v>44713</ns0:v>
+      </ns0:c>
+      <ns0:c r="B8" s="17"/>
+      <ns0:c r="C8" s="17"/>
+      <ns0:c r="D8" s="17"/>
+      <ns0:c r="E8" s="18">
+        <ns0:v>99.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="F8" s="18">
+        <ns0:v>114.87</ns0:v>
+      </ns0:c>
+      <ns0:c r="G8" s="17"/>
+      <ns0:c r="H8" s="17"/>
+      <ns0:c r="I8" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E6:$E8)^12/100^11-100</ns0:f>
+        <ns0:v>13.938422005549</ns0:v>
+      </ns0:c>
+      <ns0:c r="J8" s="3"/>
+      <ns0:c r="K8" s="3"/>
+      <ns0:c r="L8" s="3"/>
+      <ns0:c r="M8" s="3"/>
+    </ns0:row>
+    <ns0:row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A9" s="11" t="n">
+        <ns0:v>44743</ns0:v>
+      </ns0:c>
+      <ns0:c r="B9" s="17"/>
+      <ns0:c r="C9" s="17"/>
+      <ns0:c r="D9" s="17"/>
+      <ns0:c r="E9" s="18">
+        <ns0:v>99.23</ns0:v>
+      </ns0:c>
+      <ns0:c r="F9" s="18">
+        <ns0:v>113.73</ns0:v>
+      </ns0:c>
+      <ns0:c r="G9" s="17"/>
+      <ns0:c r="H9" s="17"/>
+      <ns0:c r="I9" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E7:$E9)^12/100^11-100</ns0:f>
+        <ns0:v>-3.03689051707281</ns0:v>
+      </ns0:c>
+      <ns0:c r="J9" s="3"/>
+      <ns0:c r="K9" s="3"/>
+      <ns0:c r="L9" s="3"/>
+      <ns0:c r="M9" s="3"/>
+    </ns0:row>
+    <ns0:row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A10" s="16" t="n">
+        <ns0:v>44774</ns0:v>
+      </ns0:c>
+      <ns0:c r="B10" s="17"/>
+      <ns0:c r="C10" s="17"/>
+      <ns0:c r="D10" s="17"/>
+      <ns0:c r="E10" s="18">
+        <ns0:v>99.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F10" s="18">
+        <ns0:v>112.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="G10" s="17"/>
+      <ns0:c r="H10" s="17"/>
+      <ns0:c r="I10" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E8:$E10)^12/100^11-100</ns0:f>
+        <ns0:v>-7.78738604247022</ns0:v>
+      </ns0:c>
+      <ns0:c r="J10" s="3"/>
+      <ns0:c r="K10" s="3"/>
+      <ns0:c r="L10" s="3"/>
+      <ns0:c r="M10" s="3"/>
+    </ns0:row>
+    <ns0:row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A11" s="11" t="n">
+        <ns0:v>44805</ns0:v>
+      </ns0:c>
+      <ns0:c r="B11" s="17"/>
+      <ns0:c r="C11" s="17"/>
+      <ns0:c r="D11" s="17"/>
+      <ns0:c r="E11" s="18">
+        <ns0:v>100.33</ns0:v>
+      </ns0:c>
+      <ns0:c r="F11" s="18">
+        <ns0:v>112.46</ns0:v>
+      </ns0:c>
+      <ns0:c r="G11" s="17"/>
+      <ns0:c r="H11" s="17"/>
+      <ns0:c r="I11" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E9:$E11)^12/100^11-100</ns0:f>
+        <ns0:v>-3.96602584605935</ns0:v>
+      </ns0:c>
+      <ns0:c r="J11" s="3"/>
+      <ns0:c r="K11" s="3"/>
+      <ns0:c r="L11" s="3"/>
+      <ns0:c r="M11" s="3"/>
+    </ns0:row>
+    <ns0:row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A12" s="16" t="n">
+        <ns0:v>44835</ns0:v>
+      </ns0:c>
+      <ns0:c r="B12" s="17"/>
+      <ns0:c r="C12" s="17"/>
+      <ns0:c r="D12" s="17"/>
+      <ns0:c r="E12" s="18">
+        <ns0:v>100.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="F12" s="18">
+        <ns0:v>112.17</ns0:v>
+      </ns0:c>
+      <ns0:c r="G12" s="17"/>
+      <ns0:c r="H12" s="17"/>
+      <ns0:c r="I12" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E10:$E12)^12/100^11-100</ns0:f>
+        <ns0:v>1.69299655858586</ns0:v>
+      </ns0:c>
+      <ns0:c r="J12" s="3"/>
+      <ns0:c r="K12" s="3"/>
+      <ns0:c r="L12" s="3"/>
+      <ns0:c r="M12" s="3"/>
+    </ns0:row>
+    <ns0:row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A13" s="11" t="n">
+        <ns0:v>44866</ns0:v>
+      </ns0:c>
+      <ns0:c r="B13" s="17"/>
+      <ns0:c r="C13" s="17"/>
+      <ns0:c r="D13" s="17"/>
+      <ns0:c r="E13" s="18">
+        <ns0:v>100.26</ns0:v>
+      </ns0:c>
+      <ns0:c r="F13" s="18">
+        <ns0:v>111.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G13" s="17"/>
+      <ns0:c r="H13" s="17"/>
+      <ns0:c r="I13" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E11:$E13)^12/100^11-100</ns0:f>
+        <ns0:v>5.11618978817337</ns0:v>
+      </ns0:c>
+      <ns0:c r="J13" s="3"/>
+      <ns0:c r="K13" s="3"/>
+      <ns0:c r="L13" s="3"/>
+      <ns0:c r="M13" s="3"/>
+    </ns0:row>
+    <ns0:row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A14" s="16" t="n">
+        <ns0:v>44896</ns0:v>
+      </ns0:c>
+      <ns0:c r="B14" s="17"/>
+      <ns0:c r="C14" s="17"/>
+      <ns0:c r="D14" s="17"/>
+      <ns0:c r="E14" s="18">
+        <ns0:v>100.57</ns0:v>
+      </ns0:c>
+      <ns0:c r="F14" s="18">
+        <ns0:v>111.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="G14" s="17"/>
+      <ns0:c r="H14" s="17"/>
+      <ns0:c r="I14" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E12:$E14)^12/100^11-100</ns0:f>
+        <ns0:v>6.12553306065077</ns0:v>
+      </ns0:c>
+      <ns0:c r="J14" s="3"/>
+      <ns0:c r="K14" s="3"/>
+      <ns0:c r="L14" s="3"/>
+      <ns0:c r="M14" s="3"/>
+    </ns0:row>
+    <ns0:row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A15" s="11" t="n">
+        <ns0:v>44927</ns0:v>
+      </ns0:c>
+      <ns0:c r="B15" s="17"/>
+      <ns0:c r="C15" s="17"/>
+      <ns0:c r="D15" s="17"/>
+      <ns0:c r="E15" s="18">
+        <ns0:v>101.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="F15" s="18">
+        <ns0:v>111.8</ns0:v>
+      </ns0:c>
+      <ns0:c r="G15" s="17"/>
+      <ns0:c r="H15" s="17"/>
+      <ns0:c r="I15" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E13:$E15)^12/100^11-100</ns0:f>
+        <ns0:v>8.12794364790587</ns0:v>
+      </ns0:c>
+      <ns0:c r="J15" s="3"/>
+      <ns0:c r="K15" s="3"/>
+      <ns0:c r="L15" s="3"/>
+      <ns0:c r="M15" s="3"/>
+    </ns0:row>
+    <ns0:row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A16" s="16" t="n">
+        <ns0:v>44958</ns0:v>
+      </ns0:c>
+      <ns0:c r="B16" s="19"/>
+      <ns0:c r="C16" s="19"/>
+      <ns0:c r="D16" s="19"/>
+      <ns0:c r="E16" s="20">
+        <ns0:v>100.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F16" s="20">
+        <ns0:v>111.59</ns0:v>
+      </ns0:c>
+      <ns0:c r="G16" s="19"/>
+      <ns0:c r="H16" s="19"/>
+      <ns0:c r="I16" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E14:$E16)^12/100^11-100</ns0:f>
+        <ns0:v>10.2523891898909</ns0:v>
+      </ns0:c>
+      <ns0:c r="J16" s="3"/>
+      <ns0:c r="K16" s="3"/>
+      <ns0:c r="L16" s="3"/>
+      <ns0:c r="M16" s="3"/>
+    </ns0:row>
+    <ns0:row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A17" s="11" t="n">
+        <ns0:v>44986</ns0:v>
+      </ns0:c>
+      <ns0:c r="B17" s="19"/>
+      <ns0:c r="C17" s="19"/>
+      <ns0:c r="D17" s="19"/>
+      <ns0:c r="E17" s="21">
+        <ns0:v>100.39</ns0:v>
+      </ns0:c>
+      <ns0:c r="F17" s="20">
+        <ns0:v>106.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="G17" s="19"/>
+      <ns0:c r="H17" s="19"/>
+      <ns0:c r="I17" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E15:$E17)^12/100^11-100</ns0:f>
+        <ns0:v>9.46757453632417</ns0:v>
+      </ns0:c>
+      <ns0:c r="J17" s="3"/>
+      <ns0:c r="K17" s="3"/>
+      <ns0:c r="L17" s="3"/>
+      <ns0:c r="M17" s="3"/>
+    </ns0:row>
+    <ns0:row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A18" s="16" t="n">
+        <ns0:v>45017</ns0:v>
+      </ns0:c>
+      <ns0:c r="B18" s="19"/>
+      <ns0:c r="C18" s="19"/>
+      <ns0:c r="D18" s="19"/>
+      <ns0:c r="E18" s="22">
+        <ns0:v>100.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="F18" s="20">
+        <ns0:v>103.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G18" s="19"/>
+      <ns0:c r="H18" s="19"/>
+      <ns0:c r="I18" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E16:$E18)^12/100^11-100</ns0:f>
+        <ns0:v>7.69902108971681</ns0:v>
+      </ns0:c>
+      <ns0:c r="J18" s="3"/>
+      <ns0:c r="K18" s="3"/>
+      <ns0:c r="L18" s="3"/>
+      <ns0:c r="M18" s="3"/>
+    </ns0:row>
+    <ns0:row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A19" s="11" t="n">
+        <ns0:v>45047</ns0:v>
+      </ns0:c>
+      <ns0:c r="B19" s="19"/>
+      <ns0:c r="C19" s="19"/>
+      <ns0:c r="D19" s="19"/>
+      <ns0:c r="E19" s="22">
+        <ns0:v>99.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F19" s="20">
+        <ns0:v>102.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="G19" s="19"/>
+      <ns0:c r="H19" s="19"/>
+      <ns0:c r="I19" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E17:$E19)^12/100^11-100</ns0:f>
+        <ns0:v>3.49475895939679</ns0:v>
+      </ns0:c>
+      <ns0:c r="J19" s="23"/>
+      <ns0:c r="K19" s="23"/>
+      <ns0:c r="L19" s="23"/>
+      <ns0:c r="M19" s="23"/>
+    </ns0:row>
+    <ns0:row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A20" s="16" t="n">
+        <ns0:v>45078</ns0:v>
+      </ns0:c>
+      <ns0:c r="B20" s="19"/>
+      <ns0:c r="C20" s="19"/>
+      <ns0:c r="D20" s="19"/>
+      <ns0:c r="E20" s="22">
+        <ns0:v>100.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F20" s="20">
+        <ns0:v>103.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="G20" s="19"/>
+      <ns0:c r="H20" s="19"/>
+      <ns0:c r="I20" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E18:$E20)^12/100^11-100</ns0:f>
+        <ns0:v>3.65999802881309</ns0:v>
+      </ns0:c>
+      <ns0:c r="J20" s="3"/>
+      <ns0:c r="K20" s="3"/>
+      <ns0:c r="L20" s="3"/>
+      <ns0:c r="M20" s="3"/>
+    </ns0:row>
+    <ns0:row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A21" s="11" t="n">
+        <ns0:v>45108</ns0:v>
+      </ns0:c>
+      <ns0:c r="B21" s="19"/>
+      <ns0:c r="C21" s="19"/>
+      <ns0:c r="D21" s="19"/>
+      <ns0:c r="E21" s="22">
+        <ns0:v>100.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="F21" s="20">
+        <ns0:v>105.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="G21" s="19"/>
+      <ns0:c r="H21" s="19"/>
+      <ns0:c r="I21" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E19:$E21)^12/100^11-100</ns0:f>
+        <ns0:v>2.75416684857622</ns0:v>
+      </ns0:c>
+      <ns0:c r="J21" s="3"/>
+      <ns0:c r="K21" s="3"/>
+      <ns0:c r="L21" s="3"/>
+      <ns0:c r="M21" s="3"/>
+    </ns0:row>
+    <ns0:row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A22" s="16" t="n">
+        <ns0:v>45139</ns0:v>
+      </ns0:c>
+      <ns0:c r="B22" s="19"/>
+      <ns0:c r="C22" s="19"/>
+      <ns0:c r="D22" s="19"/>
+      <ns0:c r="E22" s="22">
+        <ns0:v>99.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="F22" s="20">
+        <ns0:v>105.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="G22" s="24"/>
+      <ns0:c r="H22" s="24"/>
+      <ns0:c r="I22" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E20:$E22)^12/100^11-100</ns0:f>
+        <ns0:v>3.49475895939679</ns0:v>
+      </ns0:c>
+      <ns0:c r="J22" s="25"/>
+      <ns0:c r="K22" s="25"/>
+      <ns0:c r="L22" s="25"/>
+      <ns0:c r="M22" s="25"/>
+    </ns0:row>
+    <ns0:row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A23" s="11" t="n">
+        <ns0:v>45170</ns0:v>
+      </ns0:c>
+      <ns0:c r="B23" s="26"/>
+      <ns0:c r="C23" s="26"/>
+      <ns0:c r="D23" s="26"/>
+      <ns0:c r="E23" s="22">
+        <ns0:v>101.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F23" s="20">
+        <ns0:v>107.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="G23" s="24"/>
+      <ns0:c r="H23" s="24"/>
+      <ns0:c r="I23" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E21:$E23)^12/100^11-100</ns0:f>
+        <ns0:v>9.07709064358237</ns0:v>
+      </ns0:c>
+      <ns0:c r="J23" s="25"/>
+      <ns0:c r="K23" s="25"/>
+      <ns0:c r="L23" s="25"/>
+      <ns0:c r="M23" s="25"/>
+    </ns0:row>
+    <ns0:row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A24" s="16" t="n">
+        <ns0:v>45200</ns0:v>
+      </ns0:c>
+      <ns0:c r="B24" s="24" t="n">
+        <ns0:f aca="false">E24-0.5</ns0:f>
+        <ns0:v>99.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="C24" s="24"/>
+      <ns0:c r="D24" s="24"/>
+      <ns0:c r="E24" s="22">
+        <ns0:v>100.46</ns0:v>
+      </ns0:c>
+      <ns0:c r="F24" s="20">
+        <ns0:v>106.83</ns0:v>
+      </ns0:c>
+      <ns0:c r="G24" s="24"/>
+      <ns0:c r="H24" s="24"/>
+      <ns0:c r="I24" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E22:$E24)^12/100^11-100</ns0:f>
+        <ns0:v>8.90395244059377</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="25"/>
+      <ns0:c r="K24" s="25"/>
+      <ns0:c r="L24" s="25"/>
+      <ns0:c r="M24" s="25"/>
+    </ns0:row>
+    <ns0:row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A25" s="11" t="n">
+        <ns0:v>45231</ns0:v>
+      </ns0:c>
+      <ns0:c r="B25" s="26"/>
+      <ns0:c r="C25" s="26"/>
+      <ns0:c r="D25" s="26"/>
+      <ns0:c r="E25" s="22">
+        <ns0:v>100.74</ns0:v>
+      </ns0:c>
+      <ns0:c r="F25" s="20">
+        <ns0:v>107.34</ns0:v>
+      </ns0:c>
+      <ns0:c r="G25" s="24"/>
+      <ns0:c r="H25" s="26"/>
+      <ns0:c r="I25" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E23:$E25)^12/100^11-100</ns0:f>
+        <ns0:v>12.4595717465677</ns0:v>
+      </ns0:c>
+      <ns0:c r="J25" s="25"/>
+      <ns0:c r="K25" s="25"/>
+      <ns0:c r="L25" s="25"/>
+      <ns0:c r="M25" s="25"/>
+    </ns0:row>
+    <ns0:row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A26" s="16" t="n">
+        <ns0:v>45261</ns0:v>
+      </ns0:c>
+      <ns0:c r="B26" s="24"/>
+      <ns0:c r="C26" s="24"/>
+      <ns0:c r="D26" s="24"/>
+      <ns0:c r="E26" s="22">
+        <ns0:v>100.29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F26" s="20">
+        <ns0:v>107.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="G26" s="24"/>
+      <ns0:c r="H26" s="24"/>
+      <ns0:c r="I26" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E24:$E26)^12/100^11-100</ns0:f>
+        <ns0:v>6.12553306065077</ns0:v>
+      </ns0:c>
+      <ns0:c r="J26" s="25"/>
+      <ns0:c r="K26" s="25"/>
+      <ns0:c r="L26" s="25"/>
+      <ns0:c r="M26" s="25"/>
+    </ns0:row>
+    <ns0:row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A27" s="11" t="n">
+        <ns0:v>45292</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" s="24"/>
+      <ns0:c r="C27" s="24"/>
+      <ns0:c r="D27" s="24"/>
+      <ns0:c r="E27" s="22">
+        <ns0:v>100.87</ns0:v>
+      </ns0:c>
+      <ns0:c r="F27" s="20">
+        <ns0:v>106.77</ns0:v>
+      </ns0:c>
+      <ns0:c r="G27" s="24"/>
+      <ns0:c r="H27" s="24"/>
+      <ns0:c r="I27" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E25:$E27)^12/100^11-100</ns0:f>
+        <ns0:v>7.87040260177953</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="25"/>
+      <ns0:c r="K27" s="25"/>
+      <ns0:c r="L27" s="25"/>
+      <ns0:c r="M27" s="25"/>
+    </ns0:row>
+    <ns0:row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A28" s="16" t="n">
+        <ns0:v>45323</ns0:v>
+      </ns0:c>
+      <ns0:c r="B28" s="24"/>
+      <ns0:c r="C28" s="24"/>
+      <ns0:c r="D28" s="24"/>
+      <ns0:c r="E28" s="22">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F28" s="20">
+        <ns0:v>106.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="G28" s="24"/>
+      <ns0:c r="H28" s="24"/>
+      <ns0:c r="I28" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E26:$E28)^12/100^11-100</ns0:f>
+        <ns0:v>6.97343059130941</ns0:v>
+      </ns0:c>
+      <ns0:c r="J28" s="25"/>
+      <ns0:c r="K28" s="25"/>
+      <ns0:c r="L28" s="25"/>
+      <ns0:c r="M28" s="25"/>
+    </ns0:row>
+    <ns0:row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A29" s="11" t="n">
+        <ns0:v>45352</ns0:v>
+      </ns0:c>
+      <ns0:c r="B29" s="24"/>
+      <ns0:c r="C29" s="24"/>
+      <ns0:c r="D29" s="24"/>
+      <ns0:c r="E29" s="22">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F29" s="20">
+        <ns0:v>106.68</ns0:v>
+      </ns0:c>
+      <ns0:c r="G29" s="24"/>
+      <ns0:c r="H29" s="24"/>
+      <ns0:c r="I29" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E27:$E29)^12/100^11-100</ns0:f>
+        <ns0:v>7.99910275378316</ns0:v>
+      </ns0:c>
+      <ns0:c r="J29" s="25"/>
+      <ns0:c r="K29" s="25"/>
+      <ns0:c r="L29" s="25"/>
+      <ns0:c r="M29" s="25"/>
+    </ns0:row>
+    <ns0:row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A30" s="16" t="n">
+        <ns0:v>45383</ns0:v>
+      </ns0:c>
+      <ns0:c r="B30" s="24"/>
+      <ns0:c r="C30" s="24"/>
+      <ns0:c r="D30" s="24"/>
+      <ns0:c r="E30" s="21">
+        <ns0:v>100.38</ns0:v>
+      </ns0:c>
+      <ns0:c r="F30" s="20">
+        <ns0:v>106.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="G30" s="24"/>
+      <ns0:c r="H30" s="24"/>
+      <ns0:c r="I30" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E28:$E30)^12/100^11-100</ns0:f>
+        <ns0:v>5.91452350359876</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="25"/>
+      <ns0:c r="K30" s="25"/>
+      <ns0:c r="L30" s="25"/>
+      <ns0:c r="M30" s="25"/>
+    </ns0:row>
+    <ns0:row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A31" s="11" t="n">
+        <ns0:v>45413</ns0:v>
+      </ns0:c>
+      <ns0:c r="B31" s="24"/>
+      <ns0:c r="C31" s="24"/>
+      <ns0:c r="D31" s="24"/>
+      <ns0:c r="E31" s="21">
+        <ns0:v>100.94</ns0:v>
+      </ns0:c>
+      <ns0:c r="F31" s="20">
+        <ns0:v>107.59</ns0:v>
+      </ns0:c>
+      <ns0:c r="G31" s="24"/>
+      <ns0:c r="H31" s="24"/>
+      <ns0:c r="I31" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E29:$E31)^12/100^11-100</ns0:f>
+        <ns0:v>7.65621472911278</ns0:v>
+      </ns0:c>
+      <ns0:c r="J31" s="25"/>
+      <ns0:c r="K31" s="25"/>
+      <ns0:c r="L31" s="25"/>
+      <ns0:c r="M31" s="25"/>
+    </ns0:row>
+    <ns0:row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A32" s="16" t="n">
+        <ns0:v>45444</ns0:v>
+      </ns0:c>
+      <ns0:c r="B32" s="24"/>
+      <ns0:c r="C32" s="24"/>
+      <ns0:c r="D32" s="24"/>
+      <ns0:c r="E32" s="21">
+        <ns0:v>100.18</ns0:v>
+      </ns0:c>
+      <ns0:c r="F32" s="20">
+        <ns0:v>107.32</ns0:v>
+      </ns0:c>
+      <ns0:c r="G32" s="24"/>
+      <ns0:c r="H32" s="24"/>
+      <ns0:c r="I32" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E30:$E32)^12/100^11-100</ns0:f>
+        <ns0:v>6.16778118644996</ns0:v>
+      </ns0:c>
+      <ns0:c r="J32" s="25"/>
+      <ns0:c r="K32" s="25"/>
+      <ns0:c r="L32" s="25"/>
+      <ns0:c r="M32" s="25"/>
+    </ns0:row>
+    <ns0:row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A33" s="11" t="n">
+        <ns0:v>45474</ns0:v>
+      </ns0:c>
+      <ns0:c r="B33" s="24"/>
+      <ns0:c r="C33" s="24"/>
+      <ns0:c r="D33" s="24"/>
+      <ns0:c r="E33" s="21">
+        <ns0:v>101.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="F33" s="20">
+        <ns0:v>107.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="G33" s="24"/>
+      <ns0:c r="H33" s="24"/>
+      <ns0:c r="I33" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E31:$E33)^12/100^11-100</ns0:f>
+        <ns0:v>9.12041460123689</ns0:v>
+      </ns0:c>
+      <ns0:c r="J33" s="25"/>
+      <ns0:c r="K33" s="25"/>
+      <ns0:c r="L33" s="25"/>
+      <ns0:c r="M33" s="25"/>
+    </ns0:row>
+    <ns0:row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A34" s="16" t="n">
+        <ns0:v>45505</ns0:v>
+      </ns0:c>
+      <ns0:c r="B34" s="24"/>
+      <ns0:c r="C34" s="24"/>
+      <ns0:c r="D34" s="24"/>
+      <ns0:c r="E34" s="22">
+        <ns0:v>100.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="F34" s="20">
+        <ns0:v>108.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="G34" s="24"/>
+      <ns0:c r="H34" s="24"/>
+      <ns0:c r="I34" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E32:$E34)^12/100^11-100</ns0:f>
+        <ns0:v>5.49365770738656</ns0:v>
+      </ns0:c>
+      <ns0:c r="J34" s="25"/>
+      <ns0:c r="K34" s="25"/>
+      <ns0:c r="L34" s="25"/>
+      <ns0:c r="M34" s="25"/>
+    </ns0:row>
+    <ns0:row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A35" s="11" t="n">
+        <ns0:v>45536</ns0:v>
+      </ns0:c>
+      <ns0:c r="B35" s="24"/>
+      <ns0:c r="C35" s="24"/>
+      <ns0:c r="D35" s="24"/>
+      <ns0:c r="E35" s="21">
+        <ns0:v>100.62</ns0:v>
+      </ns0:c>
+      <ns0:c r="F35" s="20">
+        <ns0:v>106.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="G35" s="24"/>
+      <ns0:c r="H35" s="24"/>
+      <ns0:c r="I35" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E33:$E35)^12/100^11-100</ns0:f>
+        <ns0:v>7.35700662123239</ns0:v>
+      </ns0:c>
+      <ns0:c r="J35" s="25"/>
+      <ns0:c r="K35" s="25"/>
+      <ns0:c r="L35" s="25"/>
+      <ns0:c r="M35" s="25"/>
+    </ns0:row>
+    <ns0:row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A36" s="16" t="n">
+        <ns0:v>45566</ns0:v>
+      </ns0:c>
+      <ns0:c r="B36" s="24"/>
+      <ns0:c r="C36" s="24"/>
+      <ns0:c r="D36" s="24"/>
+      <ns0:c r="E36" s="22">
+        <ns0:v>101.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="F36" s="20">
+        <ns0:v>107.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G36" s="24"/>
+      <ns0:c r="H36" s="24"/>
+      <ns0:c r="I36" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E34:$E36)^12/100^11-100</ns0:f>
+        <ns0:v>7.14375346230894</ns0:v>
+      </ns0:c>
+      <ns0:c r="J36" s="25"/>
+      <ns0:c r="K36" s="25"/>
+      <ns0:c r="L36" s="25"/>
+      <ns0:c r="M36" s="25"/>
+    </ns0:row>
+    <ns0:row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A37" s="27" t="n">
+        <ns0:v>45597</ns0:v>
+      </ns0:c>
+      <ns0:c r="B37" s="28"/>
+      <ns0:c r="C37" s="28"/>
+      <ns0:c r="D37" s="28"/>
+      <ns0:c r="E37" s="29">
+        <ns0:v>101.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="F37" s="30">
+        <ns0:v>108.31</ns0:v>
+      </ns0:c>
+      <ns0:c r="G37" s="28"/>
+      <ns0:c r="H37" s="28"/>
+      <ns0:c r="I37" s="14" t="n">
+        <ns0:f aca="false">AVERAGE($E35:$E37)^12/100^11-100</ns0:f>
+        <ns0:v>13.3088674453934</ns0:v>
+      </ns0:c>
+      <ns0:c r="J37" s="25"/>
+      <ns0:c r="K37" s="25"/>
+      <ns0:c r="L37" s="25"/>
+      <ns0:c r="M37" s="25"/>
+    </ns0:row>
+    <ns0:row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A38" s="16" t="n">
+        <ns0:v>45627</ns0:v>
+      </ns0:c>
+      <ns0:c r="B38" s="31"/>
+      <ns0:c r="C38" s="31"/>
+      <ns0:c r="D38" s="31"/>
+      <ns0:c r="E38" s="22">
+        <ns0:v>100.91</ns0:v>
+      </ns0:c>
+      <ns0:c r="F38" s="20">
+        <ns0:v>108.98</ns0:v>
+      </ns0:c>
+      <ns0:c r="G38" s="32"/>
+      <ns0:c r="H38" s="31"/>
+      <ns0:c r="I38" s="24" t="n">
+        <ns0:f aca="false">AVERAGE($E36:$E38)^12/100^11-100</ns0:f>
+        <ns0:v>14.616501588559</ns0:v>
+      </ns0:c>
+      <ns0:c r="J38" s="25"/>
+      <ns0:c r="K38" s="25"/>
+      <ns0:c r="L38" s="25"/>
+      <ns0:c r="M38" s="25"/>
+    </ns0:row>
+    <ns0:row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A39" s="33" t="n">
+        <ns0:v>45658</ns0:v>
+      </ns0:c>
+      <ns0:c r="B39" s="34"/>
+      <ns0:c r="C39" s="34"/>
+      <ns0:c r="D39" s="34"/>
+      <ns0:c r="E39" s="22">
+        <ns0:v>100.84</ns0:v>
+      </ns0:c>
+      <ns0:c r="F39" s="22">
+        <ns0:v>108.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="G39" s="32"/>
+      <ns0:c r="H39" s="32"/>
+      <ns0:c r="I39" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E37:$E39)^12/100^11-100</ns0:f>
+        <ns0:v>13.8032481613878</ns0:v>
+      </ns0:c>
+      <ns0:c r="J39" s="3"/>
+      <ns0:c r="K39" s="3"/>
+      <ns0:c r="L39" s="3"/>
+      <ns0:c r="M39" s="3"/>
+    </ns0:row>
+    <ns0:row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A40" s="35" t="n">
+        <ns0:v>45689</ns0:v>
+      </ns0:c>
+      <ns0:c r="B40" s="34"/>
+      <ns0:c r="C40" s="34"/>
+      <ns0:c r="D40" s="34"/>
+      <ns0:c r="E40" s="22">
+        <ns0:v>101.34</ns0:v>
+      </ns0:c>
+      <ns0:c r="F40" s="22">
+        <ns0:v>109.83</ns0:v>
+      </ns0:c>
+      <ns0:c r="G40" s="32"/>
+      <ns0:c r="H40" s="32"/>
+      <ns0:c r="I40" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E38:$E40)^12/100^11-100</ns0:f>
+        <ns0:v>13.0848004136226</ns0:v>
+      </ns0:c>
+      <ns0:c r="J40" s="3"/>
+      <ns0:c r="K40" s="3"/>
+      <ns0:c r="L40" s="3"/>
+      <ns0:c r="M40" s="3"/>
+    </ns0:row>
+    <ns0:row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A41" s="36" t="n">
+        <ns0:v>45717</ns0:v>
+      </ns0:c>
+      <ns0:c r="B41" s="37"/>
+      <ns0:c r="C41" s="37"/>
+      <ns0:c r="D41" s="37"/>
+      <ns0:c r="E41" s="29">
+        <ns0:v>100.81</ns0:v>
+      </ns0:c>
+      <ns0:c r="F41" s="29">
+        <ns0:v>110.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="G41" s="38"/>
+      <ns0:c r="H41" s="38"/>
+      <ns0:c r="I41" s="37" t="n">
+        <ns0:f aca="false">AVERAGE($E39:$E41)^12/100^11-100</ns0:f>
+        <ns0:v>12.6378843790016</ns0:v>
+      </ns0:c>
+      <ns0:c r="J41" s="3"/>
+      <ns0:c r="K41" s="3"/>
+      <ns0:c r="L41" s="3"/>
+      <ns0:c r="M41" s="3"/>
+    </ns0:row>
+    <ns0:row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A42" s="39" t="n">
+        <ns0:v>45748</ns0:v>
+      </ns0:c>
+      <ns0:c r="B42" s="40"/>
+      <ns0:c r="C42" s="40"/>
+      <ns0:c r="D42" s="40"/>
+      <ns0:c r="E42" s="41">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F42" s="41">
+        <ns0:v>110.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="G42" s="42"/>
+      <ns0:c r="H42" s="42"/>
+      <ns0:c r="I42" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E40:$E42)^12/100^11-100</ns0:f>
+        <ns0:v>11.2627133732496</ns0:v>
+      </ns0:c>
+      <ns0:c r="J42" s="3"/>
+      <ns0:c r="K42" s="3"/>
+      <ns0:c r="L42" s="3"/>
+      <ns0:c r="M42" s="3"/>
+    </ns0:row>
+    <ns0:row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A43" s="43" t="n">
+        <ns0:v>45778</ns0:v>
+      </ns0:c>
+      <ns0:c r="B43" s="44"/>
+      <ns0:c r="C43" s="44"/>
+      <ns0:c r="D43" s="44"/>
+      <ns0:c r="E43" s="45">
+        <ns0:v>99.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="F43" s="45">
+        <ns0:v>109.19</ns0:v>
+      </ns0:c>
+      <ns0:c r="G43" s="46"/>
+      <ns0:c r="H43" s="46"/>
+      <ns0:c r="I43" s="44" t="n">
+        <ns0:f aca="false">AVERAGE($E41:$E43)^12/100^11-100</ns0:f>
+        <ns0:v>5.19996439209056</ns0:v>
+      </ns0:c>
+      <ns0:c r="J43" s="3"/>
+      <ns0:c r="K43" s="3"/>
+      <ns0:c r="L43" s="3"/>
+      <ns0:c r="M43" s="3"/>
+    </ns0:row>
+    <ns0:row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A44" s="35" t="n">
+        <ns0:v>45809</ns0:v>
+      </ns0:c>
+      <ns0:c r="B44" s="34"/>
+      <ns0:c r="C44" s="34"/>
+      <ns0:c r="D44" s="34"/>
+      <ns0:c r="E44" s="22">
+        <ns0:v>99.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="F44" s="22">
+        <ns0:v>108.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="G44" s="32"/>
+      <ns0:c r="H44" s="32"/>
+      <ns0:c r="I44" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E42:$E44)^12/100^11-100</ns0:f>
+        <ns0:v>1.69299655858586</ns0:v>
+      </ns0:c>
+      <ns0:c r="J44" s="3"/>
+      <ns0:c r="K44" s="3"/>
+      <ns0:c r="L44" s="3"/>
+      <ns0:c r="M44" s="3"/>
+    </ns0:row>
+    <ns0:row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A45" s="33" t="n">
+        <ns0:v>45839</ns0:v>
+      </ns0:c>
+      <ns0:c r="B45" s="34"/>
+      <ns0:c r="C45" s="34"/>
+      <ns0:c r="D45" s="34"/>
+      <ns0:c r="E45" s="22">
+        <ns0:v>100.36</ns0:v>
+      </ns0:c>
+      <ns0:c r="F45" s="22">
+        <ns0:v>108.19</ns0:v>
+      </ns0:c>
+      <ns0:c r="G45" s="32"/>
+      <ns0:c r="H45" s="32"/>
+      <ns0:c r="I45" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E43:$E45)^12/100^11-100</ns0:f>
+        <ns0:v>1.00459608871815</ns0:v>
+      </ns0:c>
+      <ns0:c r="J45" s="14"/>
+      <ns0:c r="K45" s="14"/>
+      <ns0:c r="L45" s="14"/>
+      <ns0:c r="M45" s="14"/>
+    </ns0:row>
+    <ns0:row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A46" s="35" t="n">
+        <ns0:v>45870</ns0:v>
+      </ns0:c>
+      <ns0:c r="B46" s="34"/>
+      <ns0:c r="C46" s="34"/>
+      <ns0:c r="D46" s="34"/>
+      <ns0:c r="E46" s="22">
+        <ns0:v>99.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F46" s="22">
+        <ns0:v>107.47</ns0:v>
+      </ns0:c>
+      <ns0:c r="G46" s="32"/>
+      <ns0:c r="H46" s="32"/>
+      <ns0:c r="I46" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E44:$E46)^12/100^11-100</ns0:f>
+        <ns0:v>-0.995429374308358</ns0:v>
+      </ns0:c>
+      <ns0:c r="J46" s="14"/>
+      <ns0:c r="K46" s="14"/>
+      <ns0:c r="L46" s="14"/>
+      <ns0:c r="M46" s="14"/>
+    </ns0:row>
+    <ns0:row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A47" s="33" t="n">
+        <ns0:v>45901</ns0:v>
+      </ns0:c>
+      <ns0:c r="B47" s="34"/>
+      <ns0:c r="C47" s="34"/>
+      <ns0:c r="D47" s="34"/>
+      <ns0:c r="E47" s="22">
+        <ns0:v>101</ns0:v>
+      </ns0:c>
+      <ns0:c r="F47" s="22">
+        <ns0:v>107.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="G47" s="32"/>
+      <ns0:c r="H47" s="32"/>
+      <ns0:c r="I47" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E45:$E47)^12/100^11-100</ns0:f>
+        <ns0:v>3.20617145915737</ns0:v>
+      </ns0:c>
+      <ns0:c r="J47" s="14"/>
+      <ns0:c r="K47" s="14"/>
+      <ns0:c r="L47" s="14"/>
+      <ns0:c r="M47" s="14"/>
+    </ns0:row>
+    <ns0:row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A48" s="35" t="n">
+        <ns0:v>45931</ns0:v>
+      </ns0:c>
+      <ns0:c r="B48" s="34"/>
+      <ns0:c r="C48" s="34"/>
+      <ns0:c r="D48" s="34"/>
+      <ns0:c r="E48" s="22">
+        <ns0:v>100.53</ns0:v>
+      </ns0:c>
+      <ns0:c r="F48" s="22">
+        <ns0:v>107.36</ns0:v>
+      </ns0:c>
+      <ns0:c r="G48" s="32"/>
+      <ns0:c r="H48" s="32"/>
+      <ns0:c r="I48" s="34" t="n">
+        <ns0:f aca="false">AVERAGE($E46:$E48)^12/100^11-100</ns0:f>
+        <ns0:v>3.90831011312588</ns0:v>
+      </ns0:c>
+      <ns0:c r="J48" s="14"/>
+      <ns0:c r="K48" s="14"/>
+      <ns0:c r="L48" s="14"/>
+      <ns0:c r="M48" s="14"/>
+    </ns0:row>
+    <ns0:row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A49" s="36" t="n">
+        <ns0:v>45962</ns0:v>
+      </ns0:c>
+      <ns0:c r="B49" s="37"/>
+      <ns0:c r="C49" s="34"/>
+      <ns0:c r="D49" s="34"/>
+      <ns0:c r="E49" s="29">
+        <ns0:v>100.15</ns0:v>
+      </ns0:c>
+      <ns0:c r="F49" s="29">
+        <ns0:v>105.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="G49" s="38"/>
+      <ns0:c r="H49" s="38"/>
+      <ns0:c r="I49" s="37" t="n">
+        <ns0:f aca="false">AVERAGE($E47:$E49)^12/100^11-100</ns0:f>
+        <ns0:v>6.93088867179823</ns0:v>
+      </ns0:c>
+      <ns0:c r="J49" s="14"/>
+      <ns0:c r="K49" s="14"/>
+      <ns0:c r="L49" s="14"/>
+      <ns0:c r="M49" s="14"/>
+    </ns0:row>
+    <ns0:row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A50" s="39" t="n">
+        <ns0:v>45992</ns0:v>
+      </ns0:c>
+      <ns0:c r="B50" s="40"/>
+      <ns0:c r="C50" s="34"/>
+      <ns0:c r="D50" s="34"/>
+      <ns0:c r="E50" s="41">
+        <ns0:v>100.29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F50" s="41">
+        <ns0:v>105.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="G50" s="42"/>
+      <ns0:c r="H50" s="42"/>
+      <ns0:c r="I50" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E48:$E50)^12/100^11-100</ns0:f>
+        <ns0:v>3.94974843103184</ns0:v>
+      </ns0:c>
+      <ns0:c r="J50" s="14"/>
+      <ns0:c r="K50" s="14"/>
+      <ns0:c r="L50" s="14"/>
+      <ns0:c r="M50" s="14"/>
+    </ns0:row>
+    <ns0:row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A51" s="43" t="n">
+        <ns0:v>46023</ns0:v>
+      </ns0:c>
+      <ns0:c r="B51" s="47"/>
+      <ns0:c r="C51" s="34" t="n">
+        <ns0:f aca="false">E51-100</ns0:f>
+        <ns0:v>1.57</ns0:v>
+      </ns0:c>
+      <ns0:c r="D51" s="34" t="n">
+        <ns0:f aca="false">F51-100</ns0:f>
+        <ns0:v>6.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="E51" s="44">
+        <ns0:v>101.57</ns0:v>
+      </ns0:c>
+      <ns0:c r="F51" s="44">
+        <ns0:f aca="false">ROUND(PRODUCT(E40:E51)/100^11,2)</ns0:f>
+        <ns0:v>106.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="G51" s="48" t="n">
+        <ns0:v>101.6</ns0:v>
+      </ns0:c>
+      <ns0:c r="H51" s="48" t="n">
+        <ns0:v>106.07</ns0:v>
+      </ns0:c>
+      <ns0:c r="I51" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E49:$E51)^12/100^11-100</ns0:f>
+        <ns0:v>8.4722085025155</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A52" s="35" t="n">
+        <ns0:v>46054</ns0:v>
+      </ns0:c>
+      <ns0:c r="B52" s="26"/>
+      <ns0:c r="C52" s="34" t="n">
+        <ns0:f aca="false">E52-100</ns0:f>
+        <ns0:v>1.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="D52" s="34" t="n">
+        <ns0:f aca="false">F52-100</ns0:f>
+        <ns0:v>5.79</ns0:v>
+      </ns0:c>
+      <ns0:c r="E52" s="34">
+        <ns0:v>101.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="F52" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E41:E52)/100^11,2)</ns0:f>
+        <ns0:v>105.79</ns0:v>
+      </ns0:c>
+      <ns0:c r="G52" s="49" t="n">
+        <ns0:v>101.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H52" s="49" t="n">
+        <ns0:v>105.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="I52" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E50:$E52)^12/100^11-100</ns0:f>
+        <ns0:v>12.6378843790016</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A53" s="33" t="n">
+        <ns0:v>46082</ns0:v>
+      </ns0:c>
+      <ns0:c r="B53" s="26"/>
+      <ns0:c r="C53" s="34" t="n">
+        <ns0:f aca="false">E53-100</ns0:f>
+        <ns0:v>0.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="D53" s="34" t="n">
+        <ns0:f aca="false">F53-100</ns0:f>
+        <ns0:v>5.51</ns0:v>
+      </ns0:c>
+      <ns0:c r="E53" s="50">
+        <ns0:v>100.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="F53" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E42:E53)/100^11,2)</ns0:f>
+        <ns0:v>105.51</ns0:v>
+      </ns0:c>
+      <ns0:c r="G53" s="49" t="n">
+        <ns0:v>100.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="H53" s="49" t="n">
+        <ns0:v>105.54</ns0:v>
+      </ns0:c>
+      <ns0:c r="I53" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E51:$E53)^12/100^11-100</ns0:f>
+        <ns0:v>13.7582228911073</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A54" s="35" t="n">
+        <ns0:v>46113</ns0:v>
+      </ns0:c>
+      <ns0:c r="B54" s="26"/>
+      <ns0:c r="C54" s="34" t="n">
+        <ns0:f aca="false">E54-100</ns0:f>
+        <ns0:v>-0.28</ns0:v>
+      </ns0:c>
+      <ns0:c r="D54" s="34" t="n">
+        <ns0:f aca="false">F54-100</ns0:f>
+        <ns0:v>4.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="E54" s="34">
+        <ns0:v>99.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="F54" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E43:E54)/100^11,2)</ns0:f>
+        <ns0:v>104.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="G54" s="49" t="n">
+        <ns0:v>99.72</ns0:v>
+      </ns0:c>
+      <ns0:c r="H54" s="49" t="n">
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="I54" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E52:$E54)^12/100^11-100</ns0:f>
+        <ns0:v>5.57770802282748</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A55" s="33" t="n">
+        <ns0:v>46143</ns0:v>
+      </ns0:c>
+      <ns0:c r="B55" s="51"/>
+      <ns0:c r="C55" s="34" t="n">
+        <ns0:f aca="false">E55-100</ns0:f>
+        <ns0:v>0.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="D55" s="34" t="n">
+        <ns0:f aca="false">F55-100</ns0:f>
+        <ns0:v>4.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="E55" s="34">
+        <ns0:v>100.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="F55" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E44:E55)/100^11,2)</ns0:f>
+        <ns0:v>104.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="G55" s="49" t="n">
+        <ns0:v>99.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="H55" s="49" t="n">
+        <ns0:v>104.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="I55" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E53:$E55)^12/100^11-100</ns0:f>
+        <ns0:v>1.4090183603949</ns0:v>
+      </ns0:c>
+      <ns0:c r="J55" s="52"/>
+      <ns0:c r="K55" s="52"/>
+      <ns0:c r="L55" s="52"/>
+      <ns0:c r="M55" s="52"/>
+    </ns0:row>
+    <ns0:row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A56" s="35" t="n">
+        <ns0:v>46174</ns0:v>
+      </ns0:c>
+      <ns0:c r="B56" s="26"/>
+      <ns0:c r="C56" s="34" t="n">
+        <ns0:f aca="false">E56-100</ns0:f>
+        <ns0:v>1.06</ns0:v>
+      </ns0:c>
+      <ns0:c r="D56" s="34" t="n">
+        <ns0:f aca="false">F56-100</ns0:f>
+        <ns0:v>5.98</ns0:v>
+      </ns0:c>
+      <ns0:c r="E56" s="34">
+        <ns0:v>101.06</ns0:v>
+      </ns0:c>
+      <ns0:c r="F56" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E45:E56)/100^11,2)</ns0:f>
+        <ns0:v>105.98</ns0:v>
+      </ns0:c>
+      <ns0:c r="G56" s="49" t="n">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="H56" s="49" t="n">
+        <ns0:v>104.7</ns0:v>
+      </ns0:c>
+      <ns0:c r="I56" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E54:$E56)^12/100^11-100</ns0:f>
+        <ns0:v>3.53604607534096</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A57" s="33" t="n">
+        <ns0:v>46204</ns0:v>
+      </ns0:c>
+      <ns0:c r="B57" s="53"/>
+      <ns0:c r="C57" s="34" t="n">
+        <ns0:f aca="false">E57-100</ns0:f>
+        <ns0:v>0.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="D57" s="34" t="n">
+        <ns0:f aca="false">F57-100</ns0:f>
+        <ns0:v>6.46</ns0:v>
+      </ns0:c>
+      <ns0:c r="E57" s="34">
+        <ns0:v>100.82</ns0:v>
+      </ns0:c>
+      <ns0:c r="F57" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E46:E57)/100^11,2)</ns0:f>
+        <ns0:v>106.46</ns0:v>
+      </ns0:c>
+      <ns0:c r="G57" s="49" t="n">
+        <ns0:v>99.9</ns0:v>
+      </ns0:c>
+      <ns0:c r="H57" s="49" t="n">
+        <ns0:v>104.22</ns0:v>
+      </ns0:c>
+      <ns0:c r="I57" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E55:$E57)^12/100^11-100</ns0:f>
+        <ns0:v>10.6906226923438</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A58" s="35" t="n">
+        <ns0:v>46235</ns0:v>
+      </ns0:c>
+      <ns0:c r="B58" s="53"/>
+      <ns0:c r="C58" s="53"/>
+      <ns0:c r="D58" s="53"/>
+      <ns0:c r="E58" s="50">
+        <ns0:v>100.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="F58" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E47:E58)/100^11,2)</ns0:f>
+        <ns0:v>107.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="G58" s="49" t="n">
+        <ns0:v>99.85</ns0:v>
+      </ns0:c>
+      <ns0:c r="H58" s="49" t="n">
+        <ns0:v>104.66</ns0:v>
+      </ns0:c>
+      <ns0:c r="I58" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E56:$E58)^12/100^11-100</ns0:f>
+        <ns0:v>10.2961408608195</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A59" s="33" t="n">
+        <ns0:v>46266</ns0:v>
+      </ns0:c>
+      <ns0:c r="B59" s="53"/>
+      <ns0:c r="C59" s="53"/>
+      <ns0:c r="D59" s="53"/>
+      <ns0:c r="E59" s="50">
+        <ns0:v>100.6</ns0:v>
+      </ns0:c>
+      <ns0:c r="F59" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E48:E59)/100^11,2)</ns0:f>
+        <ns0:v>106.78</ns0:v>
+      </ns0:c>
+      <ns0:c r="G59" s="49" t="n">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H59" s="49" t="n">
+        <ns0:v>104.09</ns0:v>
+      </ns0:c>
+      <ns0:c r="I59" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E57:$E59)^12/100^11-100</ns0:f>
+        <ns0:v>7.87040260177953</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A60" s="35" t="n">
+        <ns0:v>46296</ns0:v>
+      </ns0:c>
+      <ns0:c r="B60" s="26"/>
+      <ns0:c r="C60" s="26"/>
+      <ns0:c r="D60" s="26"/>
+      <ns0:c r="E60" s="50">
+        <ns0:v>101.33</ns0:v>
+      </ns0:c>
+      <ns0:c r="F60" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E49:E60)/100^11,2)</ns0:f>
+        <ns0:v>107.63</ns0:v>
+      </ns0:c>
+      <ns0:c r="G60" s="49" t="n">
+        <ns0:v>101.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="H60" s="49" t="n">
+        <ns0:v>104.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="I60" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E58:$E60)^12/100^11-100</ns0:f>
+        <ns0:v>7.44241677219257</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A61" s="33" t="n">
+        <ns0:v>46327</ns0:v>
+      </ns0:c>
+      <ns0:c r="B61" s="26"/>
+      <ns0:c r="C61" s="26"/>
+      <ns0:c r="D61" s="26"/>
+      <ns0:c r="E61" s="50">
+        <ns0:v>100.87</ns0:v>
+      </ns0:c>
+      <ns0:c r="F61" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E50:E61)/100^11,2)</ns0:f>
+        <ns0:v>108.4</ns0:v>
+      </ns0:c>
+      <ns0:c r="G61" s="49" t="n">
+        <ns0:v>100.3</ns0:v>
+      </ns0:c>
+      <ns0:c r="H61" s="49" t="n">
+        <ns0:v>105.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="I61" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E59:$E61)^12/100^11-100</ns0:f>
+        <ns0:v>9.38068976709832</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <ns0:c r="A62" s="35" t="n">
+        <ns0:v>46357</ns0:v>
+      </ns0:c>
+      <ns0:c r="B62" s="26"/>
+      <ns0:c r="C62" s="26"/>
+      <ns0:c r="D62" s="26"/>
+      <ns0:c r="E62" s="50">
+        <ns0:v>100.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="F62" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E51:E62)/100^11,2)</ns0:f>
+        <ns0:v>109.12</ns0:v>
+      </ns0:c>
+      <ns0:c r="G62" s="49" t="n">
+        <ns0:v>100.35</ns0:v>
+      </ns0:c>
+      <ns0:c r="H62" s="49" t="n">
+        <ns0:v>105.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="I62" s="40" t="n">
+        <ns0:f aca="false">AVERAGE($E60:$E62)^12/100^11-100</ns0:f>
+        <ns0:v>9.38068976709832</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="63" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A63" s="33" t="n">
+        <ns0:v>46388</ns0:v>
+      </ns0:c>
+      <ns0:c r="E63" s="25">
+        <ns0:v>100.99</ns0:v>
+      </ns0:c>
+      <ns0:c r="F63" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E52:E63)/100^11,2)</ns0:f>
+        <ns0:v>108.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="G63" s="54" t="n">
+        <ns0:v>100.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="H63" s="54" t="n">
+        <ns0:v>104.43</ns0:v>
+      </ns0:c>
+      <ns0:c r="I63" s="25"/>
+    </ns0:row>
+    <ns0:row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A64" s="35" t="n">
+        <ns0:v>46419</ns0:v>
+      </ns0:c>
+      <ns0:c r="E64" s="25">
+        <ns0:v>100.97</ns0:v>
+      </ns0:c>
+      <ns0:c r="F64" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E53:E64)/100^11,2)</ns0:f>
+        <ns0:v>108.36</ns0:v>
+      </ns0:c>
+      <ns0:c r="G64" s="54" t="n">
+        <ns0:v>100.65</ns0:v>
+      </ns0:c>
+      <ns0:c r="H64" s="54" t="n">
+        <ns0:v>103.97</ns0:v>
+      </ns0:c>
+      <ns0:c r="I64" s="25"/>
+    </ns0:row>
+    <ns0:row r="65" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A65" s="33" t="n">
+        <ns0:v>46447</ns0:v>
+      </ns0:c>
+      <ns0:c r="E65" s="25">
+        <ns0:v>100.78</ns0:v>
+      </ns0:c>
+      <ns0:c r="F65" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E54:E65)/100^11,2)</ns0:f>
+        <ns0:v>108.62</ns0:v>
+      </ns0:c>
+      <ns0:c r="G65" s="54" t="n">
+        <ns0:v>100.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="H65" s="54" t="n">
+        <ns0:v>103.93</ns0:v>
+      </ns0:c>
+      <ns0:c r="I65" s="25"/>
+    </ns0:row>
+    <ns0:row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A66" s="35" t="n">
+        <ns0:v>46478</ns0:v>
+      </ns0:c>
+      <ns0:c r="E66" s="25">
+        <ns0:v>100.75</ns0:v>
+      </ns0:c>
+      <ns0:c r="F66" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E55:E66)/100^11,2)</ns0:f>
+        <ns0:v>109.74</ns0:v>
+      </ns0:c>
+      <ns0:c r="G66" s="54" t="n">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H66" s="54" t="n">
+        <ns0:v>104.69</ns0:v>
+      </ns0:c>
+      <ns0:c r="I66" s="25"/>
+    </ns0:row>
+    <ns0:row r="67" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A67" s="33" t="n">
+        <ns0:v>46508</ns0:v>
+      </ns0:c>
+      <ns0:c r="E67" s="25">
+        <ns0:v>100.35</ns0:v>
+      </ns0:c>
+      <ns0:c r="F67" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E56:E67)/100^11,2)</ns0:f>
+        <ns0:v>110.03</ns0:v>
+      </ns0:c>
+      <ns0:c r="G67" s="54" t="n">
+        <ns0:v>100.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H67" s="54" t="n">
+        <ns0:v>105</ns0:v>
+      </ns0:c>
+      <ns0:c r="I67" s="25"/>
+    </ns0:row>
+    <ns0:row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A68" s="35" t="n">
+        <ns0:v>46539</ns0:v>
+      </ns0:c>
+      <ns0:c r="E68" s="25">
+        <ns0:v>100.15</ns0:v>
+      </ns0:c>
+      <ns0:c r="F68" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E57:E68)/100^11,2)</ns0:f>
+        <ns0:v>109.04</ns0:v>
+      </ns0:c>
+      <ns0:c r="G68" s="54" t="n">
+        <ns0:v>100.1</ns0:v>
+      </ns0:c>
+      <ns0:c r="H68" s="54" t="n">
+        <ns0:v>105.11</ns0:v>
+      </ns0:c>
+      <ns0:c r="I68" s="25"/>
+    </ns0:row>
+    <ns0:row r="69" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A69" s="33" t="n">
+        <ns0:v>46569</ns0:v>
+      </ns0:c>
+      <ns0:c r="E69" s="25">
+        <ns0:v>100.83</ns0:v>
+      </ns0:c>
+      <ns0:c r="F69" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E58:E69)/100^11,2)</ns0:f>
+        <ns0:v>109.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="G69" s="54" t="n">
+        <ns0:v>100.05</ns0:v>
+      </ns0:c>
+      <ns0:c r="H69" s="54" t="n">
+        <ns0:v>105.26</ns0:v>
+      </ns0:c>
+      <ns0:c r="I69" s="25"/>
+    </ns0:row>
+    <ns0:row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A70" s="35" t="n">
+        <ns0:v>46600</ns0:v>
+      </ns0:c>
+      <ns0:c r="E70" s="25">
+        <ns0:v>99.97</ns0:v>
+      </ns0:c>
+      <ns0:c r="F70" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E59:E70)/100^11,2)</ns0:f>
+        <ns0:v>108.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="G70" s="54" t="n">
+        <ns0:v>99.95</ns0:v>
+      </ns0:c>
+      <ns0:c r="H70" s="54" t="n">
+        <ns0:v>105.37</ns0:v>
+      </ns0:c>
+      <ns0:c r="I70" s="25"/>
+    </ns0:row>
+    <ns0:row r="71" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A71" s="33" t="n">
+        <ns0:v>46631</ns0:v>
+      </ns0:c>
+      <ns0:c r="E71" s="25">
+        <ns0:v>100.37</ns0:v>
+      </ns0:c>
+      <ns0:c r="F71" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E60:E71)/100^11,2)</ns0:f>
+        <ns0:v>108.64</ns0:v>
+      </ns0:c>
+      <ns0:c r="G71" s="54" t="n">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H71" s="54" t="n">
+        <ns0:v>105.37</ns0:v>
+      </ns0:c>
+      <ns0:c r="I71" s="25"/>
+    </ns0:row>
+    <ns0:row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A72" s="35" t="n">
+        <ns0:v>46661</ns0:v>
+      </ns0:c>
+      <ns0:c r="E72" s="25">
+        <ns0:v>100.41</ns0:v>
+      </ns0:c>
+      <ns0:c r="F72" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E61:E72)/100^11,2)</ns0:f>
+        <ns0:v>107.65</ns0:v>
+      </ns0:c>
+      <ns0:c r="G72" s="54" t="n">
+        <ns0:v>100.45</ns0:v>
+      </ns0:c>
+      <ns0:c r="H72" s="54" t="n">
+        <ns0:v>104.49</ns0:v>
+      </ns0:c>
+      <ns0:c r="I72" s="25"/>
+    </ns0:row>
+    <ns0:row r="73" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A73" s="33" t="n">
+        <ns0:v>46692</ns0:v>
+      </ns0:c>
+      <ns0:c r="E73" s="25">
+        <ns0:v>100.55</ns0:v>
+      </ns0:c>
+      <ns0:c r="F73" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E62:E73)/100^11,2)</ns0:f>
+        <ns0:v>107.31</ns0:v>
+      </ns0:c>
+      <ns0:c r="G73" s="54" t="n">
+        <ns0:v>100.2</ns0:v>
+      </ns0:c>
+      <ns0:c r="H73" s="54" t="n">
+        <ns0:v>104.38</ns0:v>
+      </ns0:c>
+      <ns0:c r="I73" s="25"/>
+    </ns0:row>
+    <ns0:row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A74" s="35" t="n">
+        <ns0:v>46722</ns0:v>
+      </ns0:c>
+      <ns0:c r="E74" s="25">
+        <ns0:v>100.63</ns0:v>
+      </ns0:c>
+      <ns0:c r="F74" s="34">
+        <ns0:f aca="false">ROUND(PRODUCT(E63:E74)/100^11,2)</ns0:f>
+        <ns0:v>106.96</ns0:v>
+      </ns0:c>
+      <ns0:c r="G74" s="54" t="n">
+        <ns0:v>100</ns0:v>
+      </ns0:c>
+      <ns0:c r="H74" s="54" t="n">
+        <ns0:v>104.02</ns0:v>
+      </ns0:c>
+      <ns0:c r="I74" s="25"/>
+    </ns0:row>
+    <ns0:row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A75" s="55"/>
+      <ns0:c r="E75" s="56"/>
+      <ns0:c r="F75" s="25"/>
+      <ns0:c r="G75" s="54"/>
+      <ns0:c r="H75" s="54"/>
+      <ns0:c r="I75" s="25"/>
+    </ns0:row>
+    <ns0:row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A76" s="55"/>
+      <ns0:c r="E76" s="56"/>
+      <ns0:c r="F76" s="25"/>
+      <ns0:c r="G76" s="54"/>
+      <ns0:c r="H76" s="54"/>
+      <ns0:c r="I76" s="25"/>
+    </ns0:row>
+    <ns0:row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A77" s="55"/>
+      <ns0:c r="E77" s="56"/>
+      <ns0:c r="F77" s="25"/>
+      <ns0:c r="G77" s="54"/>
+      <ns0:c r="H77" s="54"/>
+      <ns0:c r="I77" s="25"/>
+    </ns0:row>
+    <ns0:row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A78" s="55"/>
+      <ns0:c r="E78" s="56"/>
+      <ns0:c r="F78" s="25"/>
+      <ns0:c r="G78" s="54"/>
+      <ns0:c r="H78" s="54"/>
+      <ns0:c r="I78" s="25"/>
+    </ns0:row>
+    <ns0:row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="A79" s="55"/>
+      <ns0:c r="E79" s="56"/>
+      <ns0:c r="F79" s="25"/>
+      <ns0:c r="G79" s="54"/>
+      <ns0:c r="H79" s="54"/>
+      <ns0:c r="I79" s="25"/>
+    </ns0:row>
+    <ns0:row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="G81" s="14"/>
+      <ns0:c r="H81" s="14"/>
+    </ns0:row>
+    <ns0:row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <ns0:c r="G82" s="14"/>
+      <ns0:c r="H82" s="14"/>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:conditionalFormatting sqref="J23:M24">
+    <ns0:cfRule type="colorScale" priority="2">
+      <ns0:colorScale>
+        <ns0:cfvo type="min" val="0"/>
+        <ns0:cfvo type="percentile" val="50"/>
+        <ns0:cfvo type="max" val="0"/>
+        <ns0:color rgb="FF63BE7B"/>
+        <ns0:color rgb="FFFCFCFF"/>
+        <ns0:color rgb="FFF8696B"/>
+      </ns0:colorScale>
+    </ns0:cfRule>
+  </ns0:conditionalFormatting>
+  <ns0:printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <ns0:pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ns0:headerFooter differentFirst="false" differentOddEven="false">
+    <ns0:oddHeader/>
+    <ns0:oddFooter/>
+  </ns0:headerFooter>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>